<commit_message>
Made Monthly Sales Pivot Table
</commit_message>
<xml_diff>
--- a/Day 5/PivotTable_Slice_Chart.xlsx
+++ b/Day 5/PivotTable_Slice_Chart.xlsx
@@ -8,15 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DA6E53-2B0C-4BCA-83EE-137A11C3BCF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEF7F910-6601-4981-BB20-5AA782C5BC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="2" r:id="rId4"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -58,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="131">
   <si>
     <t>Sale ID</t>
   </si>
@@ -412,6 +416,45 @@
   </si>
   <si>
     <t>Month</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Aug</t>
+  </si>
+  <si>
+    <t>Sep</t>
+  </si>
+  <si>
+    <t>Oct</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Total Sale</t>
   </si>
 </sst>
 </file>
@@ -422,7 +465,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,6 +494,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -565,7 +615,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -623,12 +673,54 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" pivotButton="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="8">
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -639,6 +731,664 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="LUKE" refreshedDate="46221.998899189814" createdVersion="7" refreshedVersion="7" minRefreshableVersion="3" recordCount="40" xr:uid="{25E47070-D874-4E66-A78F-066272594201}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:J41" sheet="Sheet2"/>
+  </cacheSource>
+  <cacheFields count="10">
+    <cacheField name="Sale ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Month" numFmtId="0">
+      <sharedItems count="11">
+        <s v="Jan"/>
+        <s v="Feb"/>
+        <s v="Mar"/>
+        <s v="Apr"/>
+        <s v="May"/>
+        <s v="Jun"/>
+        <s v="Jul"/>
+        <s v="Aug"/>
+        <s v="Sep"/>
+        <s v="Oct"/>
+        <s v="Nov"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Date" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Product ID" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Region" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Qty Sold" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="20"/>
+    </cacheField>
+    <cacheField name="Product Name" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Category" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Brand" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Total Price" numFmtId="165">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="850" maxValue="770000"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="40">
+  <r>
+    <s v="S001"/>
+    <x v="0"/>
+    <s v="2024-01-05"/>
+    <s v="P001"/>
+    <s v="Dhaka"/>
+    <n v="4"/>
+    <s v="Laptop Pro"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="220000"/>
+  </r>
+  <r>
+    <s v="S002"/>
+    <x v="0"/>
+    <s v="2024-01-12"/>
+    <s v="P002"/>
+    <s v="Chittagong"/>
+    <n v="1"/>
+    <s v="Wireless Mouse"/>
+    <s v="Accessories"/>
+    <s v="TechBrand"/>
+    <n v="1200"/>
+  </r>
+  <r>
+    <s v="S003"/>
+    <x v="0"/>
+    <s v="2024-01-20"/>
+    <s v="P003"/>
+    <s v="Sylhet"/>
+    <n v="9"/>
+    <s v="Office Chair"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="135000"/>
+  </r>
+  <r>
+    <s v="S004"/>
+    <x v="0"/>
+    <s v="01/25/2024"/>
+    <s v="P004"/>
+    <s v="Rajshahi"/>
+    <n v="8"/>
+    <s v="Notebook Set"/>
+    <s v="Stationery"/>
+    <s v="WriteRight"/>
+    <n v="3600"/>
+  </r>
+  <r>
+    <s v="S005"/>
+    <x v="1"/>
+    <s v="2024-02-03"/>
+    <s v="P005"/>
+    <s v="Khulna"/>
+    <n v="8"/>
+    <s v="USB-C Hub"/>
+    <s v="Accessories"/>
+    <s v="TechBrand"/>
+    <n v="28000"/>
+  </r>
+  <r>
+    <s v="S006"/>
+    <x v="1"/>
+    <s v="2024-02-10"/>
+    <s v="P006"/>
+    <s v="Dhaka"/>
+    <n v="5"/>
+    <s v="Standing Desk"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="140000"/>
+  </r>
+  <r>
+    <s v="S006"/>
+    <x v="1"/>
+    <s v="2024-02-10"/>
+    <s v="P006"/>
+    <s v="Dhaka"/>
+    <n v="5"/>
+    <s v="Standing Desk"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="140000"/>
+  </r>
+  <r>
+    <s v="S007"/>
+    <x v="1"/>
+    <s v="2024-02-18"/>
+    <s v="P007"/>
+    <s v="Chittagong"/>
+    <n v="4"/>
+    <s v="Webcam HD"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="18000"/>
+  </r>
+  <r>
+    <s v="S009"/>
+    <x v="2"/>
+    <s v="2024-03-01"/>
+    <s v="P009"/>
+    <s v="Rajshahi"/>
+    <n v="3"/>
+    <s v="Monitor 27&quot;"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="96000"/>
+  </r>
+  <r>
+    <s v="S010"/>
+    <x v="2"/>
+    <s v="2024-03-08"/>
+    <s v="P010"/>
+    <s v="Khulna"/>
+    <n v="19"/>
+    <s v="Desk Lamp LED"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="41800"/>
+  </r>
+  <r>
+    <s v="S011"/>
+    <x v="2"/>
+    <s v="2024-03-15"/>
+    <s v="P001"/>
+    <s v="Dhaka"/>
+    <n v="14"/>
+    <s v="Laptop Pro"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="770000"/>
+  </r>
+  <r>
+    <s v="S012"/>
+    <x v="2"/>
+    <s v="2024-03-22"/>
+    <s v="P002"/>
+    <s v="Chittagong"/>
+    <n v="2"/>
+    <s v="Wireless Mouse"/>
+    <s v="Accessories"/>
+    <s v="TechBrand"/>
+    <n v="2400"/>
+  </r>
+  <r>
+    <s v="S013"/>
+    <x v="2"/>
+    <s v="03-28-2024"/>
+    <s v="P003"/>
+    <s v="Sylhet"/>
+    <n v="1"/>
+    <s v="Office Chair"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="15000"/>
+  </r>
+  <r>
+    <s v="S014"/>
+    <x v="3"/>
+    <s v="2024-04-02"/>
+    <s v="P004"/>
+    <s v="Rajshahi"/>
+    <n v="3"/>
+    <s v="Notebook Set"/>
+    <s v="Stationery"/>
+    <s v="WriteRight"/>
+    <n v="1350"/>
+  </r>
+  <r>
+    <s v="S015"/>
+    <x v="3"/>
+    <s v="2024-04-10"/>
+    <s v="P005"/>
+    <s v="Khulna"/>
+    <n v="7"/>
+    <s v="USB-C Hub"/>
+    <s v="Accessories"/>
+    <s v="TechBrand"/>
+    <n v="24500"/>
+  </r>
+  <r>
+    <s v="S017"/>
+    <x v="3"/>
+    <s v="2024-04-25"/>
+    <s v="P007"/>
+    <s v="Chittagong"/>
+    <n v="17"/>
+    <s v="Webcam HD"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="76500"/>
+  </r>
+  <r>
+    <s v="S018"/>
+    <x v="4"/>
+    <s v="2024-05-05"/>
+    <s v="P008"/>
+    <s v="Sylhet"/>
+    <n v="20"/>
+    <s v="Pen Drive 128GB"/>
+    <s v="Accessories"/>
+    <s v="StorePro"/>
+    <n v="17000"/>
+  </r>
+  <r>
+    <s v="S019"/>
+    <x v="4"/>
+    <s v="2024-05-12"/>
+    <s v="P009"/>
+    <s v="Rajshahi"/>
+    <n v="1"/>
+    <s v="Monitor 27&quot;"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="32000"/>
+  </r>
+  <r>
+    <s v="S020"/>
+    <x v="4"/>
+    <s v="2024-05-20"/>
+    <s v="P010"/>
+    <s v="Khulna"/>
+    <n v="18"/>
+    <s v="Desk Lamp LED"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="39600"/>
+  </r>
+  <r>
+    <s v="S021"/>
+    <x v="4"/>
+    <s v="2024-05-28"/>
+    <s v="P001"/>
+    <s v="Dhaka"/>
+    <n v="7"/>
+    <s v="Laptop Pro"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="385000"/>
+  </r>
+  <r>
+    <s v="S021"/>
+    <x v="4"/>
+    <s v="2024-05-28"/>
+    <s v="P001"/>
+    <s v="Dhaka"/>
+    <n v="7"/>
+    <s v="Laptop Pro"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="385000"/>
+  </r>
+  <r>
+    <s v="S022"/>
+    <x v="5"/>
+    <s v="2024-06-03"/>
+    <s v="P002"/>
+    <s v="Chittagong"/>
+    <n v="18"/>
+    <s v="Wireless Mouse"/>
+    <s v="Accessories"/>
+    <s v="TechBrand"/>
+    <n v="21600"/>
+  </r>
+  <r>
+    <s v="S023"/>
+    <x v="5"/>
+    <s v="2024-06-10"/>
+    <s v="P003"/>
+    <s v="Sylhet"/>
+    <n v="14"/>
+    <s v="Office Chair"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="210000"/>
+  </r>
+  <r>
+    <s v="S025"/>
+    <x v="5"/>
+    <s v="2024-06-25"/>
+    <s v="P005"/>
+    <s v="Khulna"/>
+    <n v="15"/>
+    <s v="USB-C Hub"/>
+    <s v="Accessories"/>
+    <s v="TechBrand"/>
+    <n v="52500"/>
+  </r>
+  <r>
+    <s v="S026"/>
+    <x v="6"/>
+    <s v="2024-07-02"/>
+    <s v="P006"/>
+    <s v="Dhaka"/>
+    <n v="19"/>
+    <s v="Standing Desk"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="532000"/>
+  </r>
+  <r>
+    <s v="S027"/>
+    <x v="6"/>
+    <s v="2024-07-10"/>
+    <s v="P007"/>
+    <s v="Chittagong"/>
+    <n v="9"/>
+    <s v="Webcam HD"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="40500"/>
+  </r>
+  <r>
+    <s v="S028"/>
+    <x v="6"/>
+    <s v="2024-07-18"/>
+    <s v="P008"/>
+    <s v="Sylhet"/>
+    <n v="1"/>
+    <s v="Pen Drive 128GB"/>
+    <s v="Accessories"/>
+    <s v="StorePro"/>
+    <n v="850"/>
+  </r>
+  <r>
+    <s v="S029"/>
+    <x v="6"/>
+    <s v="2024-07-25"/>
+    <s v="P009"/>
+    <s v="Rajshahi"/>
+    <n v="6"/>
+    <s v="Monitor 27&quot;"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="192000"/>
+  </r>
+  <r>
+    <s v="S030"/>
+    <x v="7"/>
+    <s v="2024-08-01"/>
+    <s v="P010"/>
+    <s v="Khulna"/>
+    <n v="14"/>
+    <s v="Desk Lamp LED"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="30800"/>
+  </r>
+  <r>
+    <s v="S031"/>
+    <x v="7"/>
+    <s v="2024-08-10"/>
+    <s v="P001"/>
+    <s v="Dhaka"/>
+    <n v="11"/>
+    <s v="Laptop Pro"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="605000"/>
+  </r>
+  <r>
+    <s v="S032"/>
+    <x v="7"/>
+    <s v="2024-08-18"/>
+    <s v="P002"/>
+    <s v="Chittagong"/>
+    <n v="9"/>
+    <s v="Wireless Mouse"/>
+    <s v="Accessories"/>
+    <s v="TechBrand"/>
+    <n v="10800"/>
+  </r>
+  <r>
+    <s v="S033"/>
+    <x v="7"/>
+    <s v="2024-08-25"/>
+    <s v="P003"/>
+    <s v="Sylhet"/>
+    <n v="5"/>
+    <s v="Office Chair"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="75000"/>
+  </r>
+  <r>
+    <s v="S035"/>
+    <x v="8"/>
+    <s v="2024-09-12"/>
+    <s v="P005"/>
+    <s v="Khulna"/>
+    <n v="11"/>
+    <s v="USB-C Hub"/>
+    <s v="Accessories"/>
+    <s v="TechBrand"/>
+    <n v="38500"/>
+  </r>
+  <r>
+    <s v="S036"/>
+    <x v="8"/>
+    <s v="2024-09-20"/>
+    <s v="P006"/>
+    <s v="Dhaka"/>
+    <n v="4"/>
+    <s v="Standing Desk"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="112000"/>
+  </r>
+  <r>
+    <s v="S036"/>
+    <x v="8"/>
+    <s v="2024-09-20"/>
+    <s v="P006"/>
+    <s v="Dhaka"/>
+    <n v="4"/>
+    <s v="Standing Desk"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="112000"/>
+  </r>
+  <r>
+    <s v="S037"/>
+    <x v="8"/>
+    <s v="2024-09-28"/>
+    <s v="P007"/>
+    <s v="Chittagong"/>
+    <n v="3"/>
+    <s v="Webcam HD"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="13500"/>
+  </r>
+  <r>
+    <s v="S038"/>
+    <x v="9"/>
+    <s v="2024-10-05"/>
+    <s v="P008"/>
+    <s v="Sylhet"/>
+    <n v="13"/>
+    <s v="Pen Drive 128GB"/>
+    <s v="Accessories"/>
+    <s v="StorePro"/>
+    <n v="11050"/>
+  </r>
+  <r>
+    <s v="S039"/>
+    <x v="9"/>
+    <s v="2024-10-15"/>
+    <s v="P009"/>
+    <s v="Rajshahi"/>
+    <n v="4"/>
+    <s v="Monitor 27&quot;"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="128000"/>
+  </r>
+  <r>
+    <s v="S040"/>
+    <x v="9"/>
+    <s v="2024-10-22"/>
+    <s v="P010"/>
+    <s v="Khulna"/>
+    <n v="12"/>
+    <s v="Desk Lamp LED"/>
+    <s v="Furniture"/>
+    <s v="ComfortZone"/>
+    <n v="26400"/>
+  </r>
+  <r>
+    <s v="S041"/>
+    <x v="10"/>
+    <s v="2024-11-01"/>
+    <s v="P001"/>
+    <s v="Dhaka"/>
+    <n v="12"/>
+    <s v="Laptop Pro"/>
+    <s v="Electronics"/>
+    <s v="TechBrand"/>
+    <n v="660000"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9A74C0D-44F7-4925-B9F8-FF748A2C02BC}" name="month_sales" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A3:B15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="12">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" numFmtId="165" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="12">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="7">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="5">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -838,6 +1588,125 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D581B996-E98F-4E16-A34B-9DD2229AD853}">
+  <dimension ref="A3:B15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.109375" customWidth="1"/>
+    <col min="2" max="2" width="23.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A3" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A4" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B4" s="23">
+        <v>359800</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A5" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="B5" s="23">
+        <v>326000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A6" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="23">
+        <v>925200</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A7" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B7" s="23">
+        <v>102350</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A8" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="B8" s="23">
+        <v>858600</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A9" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="23">
+        <v>284100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A10" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="23">
+        <v>765350</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A11" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="B11" s="23">
+        <v>721600</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A12" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="B12" s="23">
+        <v>276000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A13" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="B13" s="23">
+        <v>165450</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A14" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="B14" s="23">
+        <v>660000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A15" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="B15" s="23">
+        <v>5444450</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L1000"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -3557,7 +4426,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E1000"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Made Regional Sales Pivot Table
</commit_message>
<xml_diff>
--- a/Day 5/PivotTable_Slice_Chart.xlsx
+++ b/Day 5/PivotTable_Slice_Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEF7F910-6601-4981-BB20-5AA782C5BC89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF8A617-C796-477B-8AD5-CA665ED9598B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId4"/>
+    <pivotCache cacheId="3" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="131">
   <si>
     <t>Sale ID</t>
   </si>
@@ -681,7 +681,96 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="27">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <sz val="16"/>
@@ -764,7 +853,13 @@
       <sharedItems/>
     </cacheField>
     <cacheField name="Region" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="5">
+        <s v="Dhaka"/>
+        <s v="Chittagong"/>
+        <s v="Sylhet"/>
+        <s v="Rajshahi"/>
+        <s v="Khulna"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Qty Sold" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="20"/>
@@ -797,7 +892,7 @@
     <x v="0"/>
     <s v="2024-01-05"/>
     <s v="P001"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="4"/>
     <s v="Laptop Pro"/>
     <s v="Electronics"/>
@@ -809,7 +904,7 @@
     <x v="0"/>
     <s v="2024-01-12"/>
     <s v="P002"/>
-    <s v="Chittagong"/>
+    <x v="1"/>
     <n v="1"/>
     <s v="Wireless Mouse"/>
     <s v="Accessories"/>
@@ -821,7 +916,7 @@
     <x v="0"/>
     <s v="2024-01-20"/>
     <s v="P003"/>
-    <s v="Sylhet"/>
+    <x v="2"/>
     <n v="9"/>
     <s v="Office Chair"/>
     <s v="Furniture"/>
@@ -833,7 +928,7 @@
     <x v="0"/>
     <s v="01/25/2024"/>
     <s v="P004"/>
-    <s v="Rajshahi"/>
+    <x v="3"/>
     <n v="8"/>
     <s v="Notebook Set"/>
     <s v="Stationery"/>
@@ -845,7 +940,7 @@
     <x v="1"/>
     <s v="2024-02-03"/>
     <s v="P005"/>
-    <s v="Khulna"/>
+    <x v="4"/>
     <n v="8"/>
     <s v="USB-C Hub"/>
     <s v="Accessories"/>
@@ -857,7 +952,7 @@
     <x v="1"/>
     <s v="2024-02-10"/>
     <s v="P006"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="5"/>
     <s v="Standing Desk"/>
     <s v="Furniture"/>
@@ -869,7 +964,7 @@
     <x v="1"/>
     <s v="2024-02-10"/>
     <s v="P006"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="5"/>
     <s v="Standing Desk"/>
     <s v="Furniture"/>
@@ -881,7 +976,7 @@
     <x v="1"/>
     <s v="2024-02-18"/>
     <s v="P007"/>
-    <s v="Chittagong"/>
+    <x v="1"/>
     <n v="4"/>
     <s v="Webcam HD"/>
     <s v="Electronics"/>
@@ -893,7 +988,7 @@
     <x v="2"/>
     <s v="2024-03-01"/>
     <s v="P009"/>
-    <s v="Rajshahi"/>
+    <x v="3"/>
     <n v="3"/>
     <s v="Monitor 27&quot;"/>
     <s v="Electronics"/>
@@ -905,7 +1000,7 @@
     <x v="2"/>
     <s v="2024-03-08"/>
     <s v="P010"/>
-    <s v="Khulna"/>
+    <x v="4"/>
     <n v="19"/>
     <s v="Desk Lamp LED"/>
     <s v="Furniture"/>
@@ -917,7 +1012,7 @@
     <x v="2"/>
     <s v="2024-03-15"/>
     <s v="P001"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="14"/>
     <s v="Laptop Pro"/>
     <s v="Electronics"/>
@@ -929,7 +1024,7 @@
     <x v="2"/>
     <s v="2024-03-22"/>
     <s v="P002"/>
-    <s v="Chittagong"/>
+    <x v="1"/>
     <n v="2"/>
     <s v="Wireless Mouse"/>
     <s v="Accessories"/>
@@ -941,7 +1036,7 @@
     <x v="2"/>
     <s v="03-28-2024"/>
     <s v="P003"/>
-    <s v="Sylhet"/>
+    <x v="2"/>
     <n v="1"/>
     <s v="Office Chair"/>
     <s v="Furniture"/>
@@ -953,7 +1048,7 @@
     <x v="3"/>
     <s v="2024-04-02"/>
     <s v="P004"/>
-    <s v="Rajshahi"/>
+    <x v="3"/>
     <n v="3"/>
     <s v="Notebook Set"/>
     <s v="Stationery"/>
@@ -965,7 +1060,7 @@
     <x v="3"/>
     <s v="2024-04-10"/>
     <s v="P005"/>
-    <s v="Khulna"/>
+    <x v="4"/>
     <n v="7"/>
     <s v="USB-C Hub"/>
     <s v="Accessories"/>
@@ -977,7 +1072,7 @@
     <x v="3"/>
     <s v="2024-04-25"/>
     <s v="P007"/>
-    <s v="Chittagong"/>
+    <x v="1"/>
     <n v="17"/>
     <s v="Webcam HD"/>
     <s v="Electronics"/>
@@ -989,7 +1084,7 @@
     <x v="4"/>
     <s v="2024-05-05"/>
     <s v="P008"/>
-    <s v="Sylhet"/>
+    <x v="2"/>
     <n v="20"/>
     <s v="Pen Drive 128GB"/>
     <s v="Accessories"/>
@@ -1001,7 +1096,7 @@
     <x v="4"/>
     <s v="2024-05-12"/>
     <s v="P009"/>
-    <s v="Rajshahi"/>
+    <x v="3"/>
     <n v="1"/>
     <s v="Monitor 27&quot;"/>
     <s v="Electronics"/>
@@ -1013,7 +1108,7 @@
     <x v="4"/>
     <s v="2024-05-20"/>
     <s v="P010"/>
-    <s v="Khulna"/>
+    <x v="4"/>
     <n v="18"/>
     <s v="Desk Lamp LED"/>
     <s v="Furniture"/>
@@ -1025,7 +1120,7 @@
     <x v="4"/>
     <s v="2024-05-28"/>
     <s v="P001"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="7"/>
     <s v="Laptop Pro"/>
     <s v="Electronics"/>
@@ -1037,7 +1132,7 @@
     <x v="4"/>
     <s v="2024-05-28"/>
     <s v="P001"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="7"/>
     <s v="Laptop Pro"/>
     <s v="Electronics"/>
@@ -1049,7 +1144,7 @@
     <x v="5"/>
     <s v="2024-06-03"/>
     <s v="P002"/>
-    <s v="Chittagong"/>
+    <x v="1"/>
     <n v="18"/>
     <s v="Wireless Mouse"/>
     <s v="Accessories"/>
@@ -1061,7 +1156,7 @@
     <x v="5"/>
     <s v="2024-06-10"/>
     <s v="P003"/>
-    <s v="Sylhet"/>
+    <x v="2"/>
     <n v="14"/>
     <s v="Office Chair"/>
     <s v="Furniture"/>
@@ -1073,7 +1168,7 @@
     <x v="5"/>
     <s v="2024-06-25"/>
     <s v="P005"/>
-    <s v="Khulna"/>
+    <x v="4"/>
     <n v="15"/>
     <s v="USB-C Hub"/>
     <s v="Accessories"/>
@@ -1085,7 +1180,7 @@
     <x v="6"/>
     <s v="2024-07-02"/>
     <s v="P006"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="19"/>
     <s v="Standing Desk"/>
     <s v="Furniture"/>
@@ -1097,7 +1192,7 @@
     <x v="6"/>
     <s v="2024-07-10"/>
     <s v="P007"/>
-    <s v="Chittagong"/>
+    <x v="1"/>
     <n v="9"/>
     <s v="Webcam HD"/>
     <s v="Electronics"/>
@@ -1109,7 +1204,7 @@
     <x v="6"/>
     <s v="2024-07-18"/>
     <s v="P008"/>
-    <s v="Sylhet"/>
+    <x v="2"/>
     <n v="1"/>
     <s v="Pen Drive 128GB"/>
     <s v="Accessories"/>
@@ -1121,7 +1216,7 @@
     <x v="6"/>
     <s v="2024-07-25"/>
     <s v="P009"/>
-    <s v="Rajshahi"/>
+    <x v="3"/>
     <n v="6"/>
     <s v="Monitor 27&quot;"/>
     <s v="Electronics"/>
@@ -1133,7 +1228,7 @@
     <x v="7"/>
     <s v="2024-08-01"/>
     <s v="P010"/>
-    <s v="Khulna"/>
+    <x v="4"/>
     <n v="14"/>
     <s v="Desk Lamp LED"/>
     <s v="Furniture"/>
@@ -1145,7 +1240,7 @@
     <x v="7"/>
     <s v="2024-08-10"/>
     <s v="P001"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="11"/>
     <s v="Laptop Pro"/>
     <s v="Electronics"/>
@@ -1157,7 +1252,7 @@
     <x v="7"/>
     <s v="2024-08-18"/>
     <s v="P002"/>
-    <s v="Chittagong"/>
+    <x v="1"/>
     <n v="9"/>
     <s v="Wireless Mouse"/>
     <s v="Accessories"/>
@@ -1169,7 +1264,7 @@
     <x v="7"/>
     <s v="2024-08-25"/>
     <s v="P003"/>
-    <s v="Sylhet"/>
+    <x v="2"/>
     <n v="5"/>
     <s v="Office Chair"/>
     <s v="Furniture"/>
@@ -1181,7 +1276,7 @@
     <x v="8"/>
     <s v="2024-09-12"/>
     <s v="P005"/>
-    <s v="Khulna"/>
+    <x v="4"/>
     <n v="11"/>
     <s v="USB-C Hub"/>
     <s v="Accessories"/>
@@ -1193,7 +1288,7 @@
     <x v="8"/>
     <s v="2024-09-20"/>
     <s v="P006"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="4"/>
     <s v="Standing Desk"/>
     <s v="Furniture"/>
@@ -1205,7 +1300,7 @@
     <x v="8"/>
     <s v="2024-09-20"/>
     <s v="P006"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="4"/>
     <s v="Standing Desk"/>
     <s v="Furniture"/>
@@ -1217,7 +1312,7 @@
     <x v="8"/>
     <s v="2024-09-28"/>
     <s v="P007"/>
-    <s v="Chittagong"/>
+    <x v="1"/>
     <n v="3"/>
     <s v="Webcam HD"/>
     <s v="Electronics"/>
@@ -1229,7 +1324,7 @@
     <x v="9"/>
     <s v="2024-10-05"/>
     <s v="P008"/>
-    <s v="Sylhet"/>
+    <x v="2"/>
     <n v="13"/>
     <s v="Pen Drive 128GB"/>
     <s v="Accessories"/>
@@ -1241,7 +1336,7 @@
     <x v="9"/>
     <s v="2024-10-15"/>
     <s v="P009"/>
-    <s v="Rajshahi"/>
+    <x v="3"/>
     <n v="4"/>
     <s v="Monitor 27&quot;"/>
     <s v="Electronics"/>
@@ -1253,7 +1348,7 @@
     <x v="9"/>
     <s v="2024-10-22"/>
     <s v="P010"/>
-    <s v="Khulna"/>
+    <x v="4"/>
     <n v="12"/>
     <s v="Desk Lamp LED"/>
     <s v="Furniture"/>
@@ -1265,7 +1360,7 @@
     <x v="10"/>
     <s v="2024-11-01"/>
     <s v="P001"/>
-    <s v="Dhaka"/>
+    <x v="0"/>
     <n v="12"/>
     <s v="Laptop Pro"/>
     <s v="Electronics"/>
@@ -1276,7 +1371,107 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9A74C0D-44F7-4925-B9F8-FF748A2C02BC}" name="month_sales" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71DD952B-FAC6-40F9-AA5F-00E82A8D09AD}" name="PivotTable2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="D3:E9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="12">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" numFmtId="165" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="13">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="16">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="18">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9A74C0D-44F7-4925-B9F8-FF748A2C02BC}" name="month_sales" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1353,29 +1548,29 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="7">
+    <format dxfId="26">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="25">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="24">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="23">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="3">
+    <format dxfId="22">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="21">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="1">
+    <format dxfId="20">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -1589,70 +1784,114 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D581B996-E98F-4E16-A34B-9DD2229AD853}">
-  <dimension ref="A3:B15"/>
+  <dimension ref="A3:E15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.109375" customWidth="1"/>
     <col min="2" max="2" width="23.109375" customWidth="1"/>
+    <col min="4" max="4" width="19.109375" customWidth="1"/>
+    <col min="5" max="5" width="22.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="21" t="s">
         <v>117</v>
       </c>
       <c r="B3" s="22" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="D3" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A4" s="22" t="s">
         <v>118</v>
       </c>
       <c r="B4" s="23">
         <v>359800</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="D4" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="23">
+        <v>184500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="22" t="s">
         <v>119</v>
       </c>
       <c r="B5" s="23">
         <v>326000</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="D5" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="23">
+        <v>4061000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A6" s="22" t="s">
         <v>120</v>
       </c>
       <c r="B6" s="23">
         <v>925200</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="D6" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" s="23">
+        <v>282100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
         <v>121</v>
       </c>
       <c r="B7" s="23">
         <v>102350</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="D7" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="23">
+        <v>452950</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A8" s="22" t="s">
         <v>122</v>
       </c>
       <c r="B8" s="23">
         <v>858600</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="D8" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="23">
+        <v>463900</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A9" s="22" t="s">
         <v>123</v>
       </c>
       <c r="B9" s="23">
         <v>284100</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="D9" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="E9" s="23">
+        <v>5444450</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A10" s="22" t="s">
         <v>124</v>
       </c>
@@ -1660,7 +1899,7 @@
         <v>765350</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A11" s="22" t="s">
         <v>125</v>
       </c>
@@ -1668,7 +1907,7 @@
         <v>721600</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A12" s="22" t="s">
         <v>126</v>
       </c>
@@ -1676,7 +1915,7 @@
         <v>276000</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A13" s="22" t="s">
         <v>127</v>
       </c>
@@ -1684,7 +1923,7 @@
         <v>165450</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A14" s="22" t="s">
         <v>128</v>
       </c>
@@ -1692,7 +1931,7 @@
         <v>660000</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:5" ht="21" x14ac:dyDescent="0.4">
       <c r="A15" s="22" t="s">
         <v>129</v>
       </c>
@@ -1702,7 +1941,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
+  <pageSetup orientation="portrait" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Made Product based Sales Pivot Table
</commit_message>
<xml_diff>
--- a/Day 5/PivotTable_Slice_Chart.xlsx
+++ b/Day 5/PivotTable_Slice_Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF8A617-C796-477B-8AD5-CA665ED9598B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DC7259-4D0B-4B22-8495-78E82DFDC832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId4"/>
+    <pivotCache cacheId="4" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="131">
   <si>
     <t>Sale ID</t>
   </si>
@@ -681,7 +681,91 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="27">
+  <dxfs count="45">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
@@ -865,7 +949,18 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="20"/>
     </cacheField>
     <cacheField name="Product Name" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="10">
+        <s v="Laptop Pro"/>
+        <s v="Wireless Mouse"/>
+        <s v="Office Chair"/>
+        <s v="Notebook Set"/>
+        <s v="USB-C Hub"/>
+        <s v="Standing Desk"/>
+        <s v="Webcam HD"/>
+        <s v="Monitor 27&quot;"/>
+        <s v="Desk Lamp LED"/>
+        <s v="Pen Drive 128GB"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Category" numFmtId="0">
       <sharedItems/>
@@ -894,7 +989,7 @@
     <s v="P001"/>
     <x v="0"/>
     <n v="4"/>
-    <s v="Laptop Pro"/>
+    <x v="0"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="220000"/>
@@ -906,7 +1001,7 @@
     <s v="P002"/>
     <x v="1"/>
     <n v="1"/>
-    <s v="Wireless Mouse"/>
+    <x v="1"/>
     <s v="Accessories"/>
     <s v="TechBrand"/>
     <n v="1200"/>
@@ -918,7 +1013,7 @@
     <s v="P003"/>
     <x v="2"/>
     <n v="9"/>
-    <s v="Office Chair"/>
+    <x v="2"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="135000"/>
@@ -930,7 +1025,7 @@
     <s v="P004"/>
     <x v="3"/>
     <n v="8"/>
-    <s v="Notebook Set"/>
+    <x v="3"/>
     <s v="Stationery"/>
     <s v="WriteRight"/>
     <n v="3600"/>
@@ -942,7 +1037,7 @@
     <s v="P005"/>
     <x v="4"/>
     <n v="8"/>
-    <s v="USB-C Hub"/>
+    <x v="4"/>
     <s v="Accessories"/>
     <s v="TechBrand"/>
     <n v="28000"/>
@@ -954,7 +1049,7 @@
     <s v="P006"/>
     <x v="0"/>
     <n v="5"/>
-    <s v="Standing Desk"/>
+    <x v="5"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="140000"/>
@@ -966,7 +1061,7 @@
     <s v="P006"/>
     <x v="0"/>
     <n v="5"/>
-    <s v="Standing Desk"/>
+    <x v="5"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="140000"/>
@@ -978,7 +1073,7 @@
     <s v="P007"/>
     <x v="1"/>
     <n v="4"/>
-    <s v="Webcam HD"/>
+    <x v="6"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="18000"/>
@@ -990,7 +1085,7 @@
     <s v="P009"/>
     <x v="3"/>
     <n v="3"/>
-    <s v="Monitor 27&quot;"/>
+    <x v="7"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="96000"/>
@@ -1002,7 +1097,7 @@
     <s v="P010"/>
     <x v="4"/>
     <n v="19"/>
-    <s v="Desk Lamp LED"/>
+    <x v="8"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="41800"/>
@@ -1014,7 +1109,7 @@
     <s v="P001"/>
     <x v="0"/>
     <n v="14"/>
-    <s v="Laptop Pro"/>
+    <x v="0"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="770000"/>
@@ -1026,7 +1121,7 @@
     <s v="P002"/>
     <x v="1"/>
     <n v="2"/>
-    <s v="Wireless Mouse"/>
+    <x v="1"/>
     <s v="Accessories"/>
     <s v="TechBrand"/>
     <n v="2400"/>
@@ -1038,7 +1133,7 @@
     <s v="P003"/>
     <x v="2"/>
     <n v="1"/>
-    <s v="Office Chair"/>
+    <x v="2"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="15000"/>
@@ -1050,7 +1145,7 @@
     <s v="P004"/>
     <x v="3"/>
     <n v="3"/>
-    <s v="Notebook Set"/>
+    <x v="3"/>
     <s v="Stationery"/>
     <s v="WriteRight"/>
     <n v="1350"/>
@@ -1062,7 +1157,7 @@
     <s v="P005"/>
     <x v="4"/>
     <n v="7"/>
-    <s v="USB-C Hub"/>
+    <x v="4"/>
     <s v="Accessories"/>
     <s v="TechBrand"/>
     <n v="24500"/>
@@ -1074,7 +1169,7 @@
     <s v="P007"/>
     <x v="1"/>
     <n v="17"/>
-    <s v="Webcam HD"/>
+    <x v="6"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="76500"/>
@@ -1086,7 +1181,7 @@
     <s v="P008"/>
     <x v="2"/>
     <n v="20"/>
-    <s v="Pen Drive 128GB"/>
+    <x v="9"/>
     <s v="Accessories"/>
     <s v="StorePro"/>
     <n v="17000"/>
@@ -1098,7 +1193,7 @@
     <s v="P009"/>
     <x v="3"/>
     <n v="1"/>
-    <s v="Monitor 27&quot;"/>
+    <x v="7"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="32000"/>
@@ -1110,7 +1205,7 @@
     <s v="P010"/>
     <x v="4"/>
     <n v="18"/>
-    <s v="Desk Lamp LED"/>
+    <x v="8"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="39600"/>
@@ -1122,7 +1217,7 @@
     <s v="P001"/>
     <x v="0"/>
     <n v="7"/>
-    <s v="Laptop Pro"/>
+    <x v="0"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="385000"/>
@@ -1134,7 +1229,7 @@
     <s v="P001"/>
     <x v="0"/>
     <n v="7"/>
-    <s v="Laptop Pro"/>
+    <x v="0"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="385000"/>
@@ -1146,7 +1241,7 @@
     <s v="P002"/>
     <x v="1"/>
     <n v="18"/>
-    <s v="Wireless Mouse"/>
+    <x v="1"/>
     <s v="Accessories"/>
     <s v="TechBrand"/>
     <n v="21600"/>
@@ -1158,7 +1253,7 @@
     <s v="P003"/>
     <x v="2"/>
     <n v="14"/>
-    <s v="Office Chair"/>
+    <x v="2"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="210000"/>
@@ -1170,7 +1265,7 @@
     <s v="P005"/>
     <x v="4"/>
     <n v="15"/>
-    <s v="USB-C Hub"/>
+    <x v="4"/>
     <s v="Accessories"/>
     <s v="TechBrand"/>
     <n v="52500"/>
@@ -1182,7 +1277,7 @@
     <s v="P006"/>
     <x v="0"/>
     <n v="19"/>
-    <s v="Standing Desk"/>
+    <x v="5"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="532000"/>
@@ -1194,7 +1289,7 @@
     <s v="P007"/>
     <x v="1"/>
     <n v="9"/>
-    <s v="Webcam HD"/>
+    <x v="6"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="40500"/>
@@ -1206,7 +1301,7 @@
     <s v="P008"/>
     <x v="2"/>
     <n v="1"/>
-    <s v="Pen Drive 128GB"/>
+    <x v="9"/>
     <s v="Accessories"/>
     <s v="StorePro"/>
     <n v="850"/>
@@ -1218,7 +1313,7 @@
     <s v="P009"/>
     <x v="3"/>
     <n v="6"/>
-    <s v="Monitor 27&quot;"/>
+    <x v="7"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="192000"/>
@@ -1230,7 +1325,7 @@
     <s v="P010"/>
     <x v="4"/>
     <n v="14"/>
-    <s v="Desk Lamp LED"/>
+    <x v="8"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="30800"/>
@@ -1242,7 +1337,7 @@
     <s v="P001"/>
     <x v="0"/>
     <n v="11"/>
-    <s v="Laptop Pro"/>
+    <x v="0"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="605000"/>
@@ -1254,7 +1349,7 @@
     <s v="P002"/>
     <x v="1"/>
     <n v="9"/>
-    <s v="Wireless Mouse"/>
+    <x v="1"/>
     <s v="Accessories"/>
     <s v="TechBrand"/>
     <n v="10800"/>
@@ -1266,7 +1361,7 @@
     <s v="P003"/>
     <x v="2"/>
     <n v="5"/>
-    <s v="Office Chair"/>
+    <x v="2"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="75000"/>
@@ -1278,7 +1373,7 @@
     <s v="P005"/>
     <x v="4"/>
     <n v="11"/>
-    <s v="USB-C Hub"/>
+    <x v="4"/>
     <s v="Accessories"/>
     <s v="TechBrand"/>
     <n v="38500"/>
@@ -1290,7 +1385,7 @@
     <s v="P006"/>
     <x v="0"/>
     <n v="4"/>
-    <s v="Standing Desk"/>
+    <x v="5"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="112000"/>
@@ -1302,7 +1397,7 @@
     <s v="P006"/>
     <x v="0"/>
     <n v="4"/>
-    <s v="Standing Desk"/>
+    <x v="5"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="112000"/>
@@ -1314,7 +1409,7 @@
     <s v="P007"/>
     <x v="1"/>
     <n v="3"/>
-    <s v="Webcam HD"/>
+    <x v="6"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="13500"/>
@@ -1326,7 +1421,7 @@
     <s v="P008"/>
     <x v="2"/>
     <n v="13"/>
-    <s v="Pen Drive 128GB"/>
+    <x v="9"/>
     <s v="Accessories"/>
     <s v="StorePro"/>
     <n v="11050"/>
@@ -1338,7 +1433,7 @@
     <s v="P009"/>
     <x v="3"/>
     <n v="4"/>
-    <s v="Monitor 27&quot;"/>
+    <x v="7"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="128000"/>
@@ -1350,7 +1445,7 @@
     <s v="P010"/>
     <x v="4"/>
     <n v="12"/>
-    <s v="Desk Lamp LED"/>
+    <x v="8"/>
     <s v="Furniture"/>
     <s v="ComfortZone"/>
     <n v="26400"/>
@@ -1362,7 +1457,7 @@
     <s v="P001"/>
     <x v="0"/>
     <n v="12"/>
-    <s v="Laptop Pro"/>
+    <x v="0"/>
     <s v="Electronics"/>
     <s v="TechBrand"/>
     <n v="660000"/>
@@ -1371,7 +1466,136 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71DD952B-FAC6-40F9-AA5F-00E82A8D09AD}" name="PivotTable2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FC6400F2-21E4-469F-9AF0-F99BBDA61EFA}" name="PivotTable3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="G3:H14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="12">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="11">
+        <item x="8"/>
+        <item x="0"/>
+        <item x="7"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="9"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="6"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" numFmtId="165" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="12">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
+    </format>
+    <format dxfId="16">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71DD952B-FAC6-40F9-AA5F-00E82A8D09AD}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="D3:E9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1439,22 +1663,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="13">
+    <format dxfId="31">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="32">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="33">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="34">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="36">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -1470,8 +1694,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9A74C0D-44F7-4925-B9F8-FF748A2C02BC}" name="month_sales" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9A74C0D-44F7-4925-B9F8-FF748A2C02BC}" name="month_sales" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1548,29 +1772,29 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="26">
+    <format dxfId="44">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="25">
+    <format dxfId="43">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="24">
+    <format dxfId="42">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="23">
+    <format dxfId="41">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="22">
+    <format dxfId="40">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="21">
+    <format dxfId="39">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="38">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -1784,16 +2008,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D581B996-E98F-4E16-A34B-9DD2229AD853}">
-  <dimension ref="A3:E15"/>
+  <dimension ref="A3:H19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.109375" customWidth="1"/>
     <col min="2" max="2" width="23.109375" customWidth="1"/>
     <col min="4" max="4" width="19.109375" customWidth="1"/>
     <col min="5" max="5" width="22.77734375" customWidth="1"/>
+    <col min="7" max="7" width="23.77734375" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" customWidth="1"/>
+    <col min="9" max="9" width="19.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="21" t="s">
         <v>117</v>
       </c>
@@ -1806,8 +2033,14 @@
       <c r="E3" s="22" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G3" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A4" s="22" t="s">
         <v>118</v>
       </c>
@@ -1820,8 +2053,14 @@
       <c r="E4" s="23">
         <v>184500</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G4" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="H4" s="23">
+        <v>138600</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="22" t="s">
         <v>119</v>
       </c>
@@ -1834,8 +2073,14 @@
       <c r="E5" s="23">
         <v>4061000</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G5" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="23">
+        <v>3025000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A6" s="22" t="s">
         <v>120</v>
       </c>
@@ -1848,8 +2093,14 @@
       <c r="E6" s="23">
         <v>282100</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G6" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="23">
+        <v>448000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
         <v>121</v>
       </c>
@@ -1862,8 +2113,14 @@
       <c r="E7" s="23">
         <v>452950</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G7" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="23">
+        <v>4950</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A8" s="22" t="s">
         <v>122</v>
       </c>
@@ -1876,8 +2133,14 @@
       <c r="E8" s="23">
         <v>463900</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G8" s="22" t="s">
+        <v>25</v>
+      </c>
+      <c r="H8" s="23">
+        <v>435000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A9" s="22" t="s">
         <v>123</v>
       </c>
@@ -1890,48 +2153,84 @@
       <c r="E9" s="23">
         <v>5444450</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G9" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="H9" s="23">
+        <v>28900</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A10" s="22" t="s">
         <v>124</v>
       </c>
       <c r="B10" s="23">
         <v>765350</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G10" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="H10" s="23">
+        <v>1036000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A11" s="22" t="s">
         <v>125</v>
       </c>
       <c r="B11" s="23">
         <v>721600</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G11" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="23">
+        <v>143500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A12" s="22" t="s">
         <v>126</v>
       </c>
       <c r="B12" s="23">
         <v>276000</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G12" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="H12" s="23">
+        <v>148500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A13" s="22" t="s">
         <v>127</v>
       </c>
       <c r="B13" s="23">
         <v>165450</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G13" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" s="23">
+        <v>36000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A14" s="22" t="s">
         <v>128</v>
       </c>
       <c r="B14" s="23">
         <v>660000</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="21" x14ac:dyDescent="0.4">
+      <c r="G14" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="H14" s="23">
+        <v>5444450</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="21" x14ac:dyDescent="0.4">
       <c r="A15" s="22" t="s">
         <v>129</v>
       </c>
@@ -1939,9 +2238,13 @@
         <v>5444450</v>
       </c>
     </row>
+    <row r="16" spans="1:8" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="17" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="18" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="19" ht="21" x14ac:dyDescent="0.4"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Made Category based Sales Pivot Table
</commit_message>
<xml_diff>
--- a/Day 5/PivotTable_Slice_Chart.xlsx
+++ b/Day 5/PivotTable_Slice_Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1DC7259-4D0B-4B22-8495-78E82DFDC832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E45CA0-DD2A-44DC-A4D7-3CF1910DD898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId4"/>
+    <pivotCache cacheId="5" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="131">
   <si>
     <t>Sale ID</t>
   </si>
@@ -681,7 +681,91 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="45">
+  <dxfs count="63">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
@@ -963,7 +1047,12 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Category" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="4">
+        <s v="Electronics"/>
+        <s v="Accessories"/>
+        <s v="Furniture"/>
+        <s v="Stationery"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Brand" numFmtId="0">
       <sharedItems/>
@@ -990,7 +1079,7 @@
     <x v="0"/>
     <n v="4"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="220000"/>
   </r>
@@ -1002,7 +1091,7 @@
     <x v="1"/>
     <n v="1"/>
     <x v="1"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="TechBrand"/>
     <n v="1200"/>
   </r>
@@ -1014,7 +1103,7 @@
     <x v="2"/>
     <n v="9"/>
     <x v="2"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="135000"/>
   </r>
@@ -1026,7 +1115,7 @@
     <x v="3"/>
     <n v="8"/>
     <x v="3"/>
-    <s v="Stationery"/>
+    <x v="3"/>
     <s v="WriteRight"/>
     <n v="3600"/>
   </r>
@@ -1038,7 +1127,7 @@
     <x v="4"/>
     <n v="8"/>
     <x v="4"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="TechBrand"/>
     <n v="28000"/>
   </r>
@@ -1050,7 +1139,7 @@
     <x v="0"/>
     <n v="5"/>
     <x v="5"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="140000"/>
   </r>
@@ -1062,7 +1151,7 @@
     <x v="0"/>
     <n v="5"/>
     <x v="5"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="140000"/>
   </r>
@@ -1074,7 +1163,7 @@
     <x v="1"/>
     <n v="4"/>
     <x v="6"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="18000"/>
   </r>
@@ -1086,7 +1175,7 @@
     <x v="3"/>
     <n v="3"/>
     <x v="7"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="96000"/>
   </r>
@@ -1098,7 +1187,7 @@
     <x v="4"/>
     <n v="19"/>
     <x v="8"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="41800"/>
   </r>
@@ -1110,7 +1199,7 @@
     <x v="0"/>
     <n v="14"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="770000"/>
   </r>
@@ -1122,7 +1211,7 @@
     <x v="1"/>
     <n v="2"/>
     <x v="1"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="TechBrand"/>
     <n v="2400"/>
   </r>
@@ -1134,7 +1223,7 @@
     <x v="2"/>
     <n v="1"/>
     <x v="2"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="15000"/>
   </r>
@@ -1146,7 +1235,7 @@
     <x v="3"/>
     <n v="3"/>
     <x v="3"/>
-    <s v="Stationery"/>
+    <x v="3"/>
     <s v="WriteRight"/>
     <n v="1350"/>
   </r>
@@ -1158,7 +1247,7 @@
     <x v="4"/>
     <n v="7"/>
     <x v="4"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="TechBrand"/>
     <n v="24500"/>
   </r>
@@ -1170,7 +1259,7 @@
     <x v="1"/>
     <n v="17"/>
     <x v="6"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="76500"/>
   </r>
@@ -1182,7 +1271,7 @@
     <x v="2"/>
     <n v="20"/>
     <x v="9"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="StorePro"/>
     <n v="17000"/>
   </r>
@@ -1194,7 +1283,7 @@
     <x v="3"/>
     <n v="1"/>
     <x v="7"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="32000"/>
   </r>
@@ -1206,7 +1295,7 @@
     <x v="4"/>
     <n v="18"/>
     <x v="8"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="39600"/>
   </r>
@@ -1218,7 +1307,7 @@
     <x v="0"/>
     <n v="7"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="385000"/>
   </r>
@@ -1230,7 +1319,7 @@
     <x v="0"/>
     <n v="7"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="385000"/>
   </r>
@@ -1242,7 +1331,7 @@
     <x v="1"/>
     <n v="18"/>
     <x v="1"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="TechBrand"/>
     <n v="21600"/>
   </r>
@@ -1254,7 +1343,7 @@
     <x v="2"/>
     <n v="14"/>
     <x v="2"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="210000"/>
   </r>
@@ -1266,7 +1355,7 @@
     <x v="4"/>
     <n v="15"/>
     <x v="4"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="TechBrand"/>
     <n v="52500"/>
   </r>
@@ -1278,7 +1367,7 @@
     <x v="0"/>
     <n v="19"/>
     <x v="5"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="532000"/>
   </r>
@@ -1290,7 +1379,7 @@
     <x v="1"/>
     <n v="9"/>
     <x v="6"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="40500"/>
   </r>
@@ -1302,7 +1391,7 @@
     <x v="2"/>
     <n v="1"/>
     <x v="9"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="StorePro"/>
     <n v="850"/>
   </r>
@@ -1314,7 +1403,7 @@
     <x v="3"/>
     <n v="6"/>
     <x v="7"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="192000"/>
   </r>
@@ -1326,7 +1415,7 @@
     <x v="4"/>
     <n v="14"/>
     <x v="8"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="30800"/>
   </r>
@@ -1338,7 +1427,7 @@
     <x v="0"/>
     <n v="11"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="605000"/>
   </r>
@@ -1350,7 +1439,7 @@
     <x v="1"/>
     <n v="9"/>
     <x v="1"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="TechBrand"/>
     <n v="10800"/>
   </r>
@@ -1362,7 +1451,7 @@
     <x v="2"/>
     <n v="5"/>
     <x v="2"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="75000"/>
   </r>
@@ -1374,7 +1463,7 @@
     <x v="4"/>
     <n v="11"/>
     <x v="4"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="TechBrand"/>
     <n v="38500"/>
   </r>
@@ -1386,7 +1475,7 @@
     <x v="0"/>
     <n v="4"/>
     <x v="5"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="112000"/>
   </r>
@@ -1398,7 +1487,7 @@
     <x v="0"/>
     <n v="4"/>
     <x v="5"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="112000"/>
   </r>
@@ -1410,7 +1499,7 @@
     <x v="1"/>
     <n v="3"/>
     <x v="6"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="13500"/>
   </r>
@@ -1422,7 +1511,7 @@
     <x v="2"/>
     <n v="13"/>
     <x v="9"/>
-    <s v="Accessories"/>
+    <x v="1"/>
     <s v="StorePro"/>
     <n v="11050"/>
   </r>
@@ -1434,7 +1523,7 @@
     <x v="3"/>
     <n v="4"/>
     <x v="7"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="128000"/>
   </r>
@@ -1446,7 +1535,7 @@
     <x v="4"/>
     <n v="12"/>
     <x v="8"/>
-    <s v="Furniture"/>
+    <x v="2"/>
     <s v="ComfortZone"/>
     <n v="26400"/>
   </r>
@@ -1458,7 +1547,7 @@
     <x v="0"/>
     <n v="12"/>
     <x v="0"/>
-    <s v="Electronics"/>
+    <x v="0"/>
     <s v="TechBrand"/>
     <n v="660000"/>
   </r>
@@ -1466,7 +1555,112 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FC6400F2-21E4-469F-9AF0-F99BBDA61EFA}" name="PivotTable3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48B9EF5A-3213-4D38-979A-0805F2D584A7}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="J3:K8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="10">
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="12">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" numFmtId="165" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="12">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
+    </format>
+    <format dxfId="16">
+      <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FC6400F2-21E4-469F-9AF0-F99BBDA61EFA}" name="PivotTable3" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="G3:H14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1563,22 +1757,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="12">
+    <format dxfId="30">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="31">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="32">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="33">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="34">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="35">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -1594,8 +1788,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71DD952B-FAC6-40F9-AA5F-00E82A8D09AD}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71DD952B-FAC6-40F9-AA5F-00E82A8D09AD}" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="D3:E9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1663,22 +1857,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="31">
+    <format dxfId="49">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="50">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="51">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="34">
+    <format dxfId="52">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="53">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="36">
+    <format dxfId="54">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -1694,8 +1888,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9A74C0D-44F7-4925-B9F8-FF748A2C02BC}" name="month_sales" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9A74C0D-44F7-4925-B9F8-FF748A2C02BC}" name="month_sales" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:B15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1772,29 +1966,29 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="44">
+    <format dxfId="62">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="43">
+    <format dxfId="61">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="42">
+    <format dxfId="60">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="41">
+    <format dxfId="59">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="40">
+    <format dxfId="58">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="39">
+    <format dxfId="57">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="38">
+    <format dxfId="56">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -2008,7 +2202,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D581B996-E98F-4E16-A34B-9DD2229AD853}">
-  <dimension ref="A3:H19"/>
+  <dimension ref="A3:K19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.109375" customWidth="1"/>
@@ -2017,10 +2211,13 @@
     <col min="5" max="5" width="22.77734375" customWidth="1"/>
     <col min="7" max="7" width="23.77734375" customWidth="1"/>
     <col min="8" max="8" width="21.5546875" customWidth="1"/>
-    <col min="9" max="9" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.21875" customWidth="1"/>
+    <col min="10" max="10" width="17.88671875" customWidth="1"/>
+    <col min="11" max="11" width="21.109375" customWidth="1"/>
+    <col min="12" max="12" width="19.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A3" s="21" t="s">
         <v>117</v>
       </c>
@@ -2039,8 +2236,14 @@
       <c r="H3" s="22" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="J3" s="21" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A4" s="22" t="s">
         <v>118</v>
       </c>
@@ -2059,8 +2262,14 @@
       <c r="H4" s="23">
         <v>138600</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="J4" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="23">
+        <v>208400</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A5" s="22" t="s">
         <v>119</v>
       </c>
@@ -2079,8 +2288,14 @@
       <c r="H5" s="23">
         <v>3025000</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="J5" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="23">
+        <v>3621500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A6" s="22" t="s">
         <v>120</v>
       </c>
@@ -2099,8 +2314,14 @@
       <c r="H6" s="23">
         <v>448000</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="J6" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="23">
+        <v>1609600</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A7" s="22" t="s">
         <v>121</v>
       </c>
@@ -2119,8 +2340,14 @@
       <c r="H7" s="23">
         <v>4950</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="J7" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" s="23">
+        <v>4950</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A8" s="22" t="s">
         <v>122</v>
       </c>
@@ -2139,8 +2366,14 @@
       <c r="H8" s="23">
         <v>435000</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+      <c r="J8" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="K8" s="23">
+        <v>5444450</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A9" s="22" t="s">
         <v>123</v>
       </c>
@@ -2160,7 +2393,7 @@
         <v>28900</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A10" s="22" t="s">
         <v>124</v>
       </c>
@@ -2174,7 +2407,7 @@
         <v>1036000</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A11" s="22" t="s">
         <v>125</v>
       </c>
@@ -2188,7 +2421,7 @@
         <v>143500</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A12" s="22" t="s">
         <v>126</v>
       </c>
@@ -2202,7 +2435,7 @@
         <v>148500</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A13" s="22" t="s">
         <v>127</v>
       </c>
@@ -2216,7 +2449,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A14" s="22" t="s">
         <v>128</v>
       </c>
@@ -2230,7 +2463,7 @@
         <v>5444450</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="21" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A15" s="22" t="s">
         <v>129</v>
       </c>
@@ -2238,13 +2471,13 @@
         <v>5444450</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="16" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
     <row r="17" ht="21" x14ac:dyDescent="0.4"/>
     <row r="18" ht="21" x14ac:dyDescent="0.4"/>
     <row r="19" ht="21" x14ac:dyDescent="0.4"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Slicer is added for Month and Connected
</commit_message>
<xml_diff>
--- a/Day 5/PivotTable_Slice_Chart.xlsx
+++ b/Day 5/PivotTable_Slice_Chart.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25128"/>
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98E45CA0-DD2A-44DC-A4D7-3CF1910DD898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F11FF63-DE69-4BF0-B1FB-95AAD218D66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,11 +17,22 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="Slicer_Month">#N/A</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="5" r:id="rId4"/>
   </pivotCaches>
   <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
+      <x14:slicerCaches>
+        <x14:slicerCache r:id="rId5"/>
+      </x14:slicerCaches>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -681,7 +692,7 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="63">
+  <dxfs count="376">
     <dxf>
       <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
@@ -795,6 +806,11 @@
       </font>
     </dxf>
     <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
@@ -918,6 +934,1466 @@
       <font>
         <sz val="16"/>
       </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
       <font>
@@ -988,6 +2464,89 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>7620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>419100</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>74295</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Month">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B80171C-3EE8-FFC4-41BE-087637E193C1}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Month"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="12611100" y="373380"/>
+              <a:ext cx="1828800" cy="2466975"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1063,7 +2622,7 @@
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
+      <x14:pivotCacheDefinition pivotCacheId="1167224161"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -1555,7 +3114,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48B9EF5A-3213-4D38-979A-0805F2D584A7}" name="PivotTable4" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48B9EF5A-3213-4D38-979A-0805F2D584A7}" name="productcategory_sales" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="J3:K8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1628,22 +3187,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="12">
+    <format dxfId="351">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="352">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="14">
+    <format dxfId="353">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="354">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="355">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="356">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -1660,7 +3219,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FC6400F2-21E4-469F-9AF0-F99BBDA61EFA}" name="PivotTable3" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FC6400F2-21E4-469F-9AF0-F99BBDA61EFA}" name="productname_sales" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="G3:H14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1757,22 +3316,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="30">
+    <format dxfId="357">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="31">
+    <format dxfId="358">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="32">
+    <format dxfId="359">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="33">
+    <format dxfId="360">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="34">
+    <format dxfId="361">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="35">
+    <format dxfId="362">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -1789,7 +3348,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71DD952B-FAC6-40F9-AA5F-00E82A8D09AD}" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71DD952B-FAC6-40F9-AA5F-00E82A8D09AD}" name="region_sales" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="D3:E9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
@@ -1857,22 +3416,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="49">
+    <format dxfId="363">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="50">
+    <format dxfId="364">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="51">
+    <format dxfId="365">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="52">
+    <format dxfId="366">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="53">
+    <format dxfId="367">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="54">
+    <format dxfId="368">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -1966,29 +3525,29 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="62">
+    <format dxfId="375">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="61">
+    <format dxfId="374">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="60">
+    <format dxfId="373">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="59">
+    <format dxfId="372">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="58">
+    <format dxfId="371">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="57">
+    <format dxfId="370">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="56">
+    <format dxfId="369">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -2002,6 +3561,40 @@
     </ext>
   </extLst>
 </pivotTableDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Month" xr10:uid="{2FB4EC41-1CBD-45D7-90E0-038E93BAD8D3}" sourceName="Month">
+  <pivotTables>
+    <pivotTable tabId="4" name="month_sales"/>
+    <pivotTable tabId="4" name="productcategory_sales"/>
+    <pivotTable tabId="4" name="productname_sales"/>
+    <pivotTable tabId="4" name="region_sales"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1167224161">
+      <items count="11">
+        <i x="0" s="1"/>
+        <i x="1" s="1"/>
+        <i x="2" s="1"/>
+        <i x="3" s="1"/>
+        <i x="4" s="1"/>
+        <i x="5" s="1"/>
+        <i x="6" s="1"/>
+        <i x="7" s="1"/>
+        <i x="8" s="1"/>
+        <i x="9" s="1"/>
+        <i x="10" s="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
+<slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
+  <slicer name="Month" xr10:uid="{8F227F2F-9E99-497F-B577-006C74605616}" cache="Slicer_Month" caption="Month" rowHeight="234950"/>
+</slicers>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2205,16 +3798,16 @@
   <dimension ref="A3:K19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.109375" customWidth="1"/>
-    <col min="2" max="2" width="23.109375" customWidth="1"/>
-    <col min="4" max="4" width="19.109375" customWidth="1"/>
-    <col min="5" max="5" width="22.77734375" customWidth="1"/>
-    <col min="7" max="7" width="23.77734375" customWidth="1"/>
-    <col min="8" max="8" width="21.5546875" customWidth="1"/>
+    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.21875" customWidth="1"/>
-    <col min="10" max="10" width="17.88671875" customWidth="1"/>
-    <col min="11" max="11" width="21.109375" customWidth="1"/>
-    <col min="12" max="12" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:11" ht="21" x14ac:dyDescent="0.4">
@@ -2478,6 +4071,14 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId5"/>
+  <drawing r:id="rId6"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
+      <x14:slicerList>
+        <x14:slicer r:id="rId7"/>
+      </x14:slicerList>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Other Slicers are added
</commit_message>
<xml_diff>
--- a/Day 5/PivotTable_Slice_Chart.xlsx
+++ b/Day 5/PivotTable_Slice_Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Data Analycis\Data Analytics Practice\Day 5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F11FF63-DE69-4BF0-B1FB-95AAD218D66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B465BE3D-148A-48DD-B846-6F9D18BE841B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,10 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="Slicer_Category">#N/A</definedName>
     <definedName name="Slicer_Month">#N/A</definedName>
+    <definedName name="Slicer_Product_Name">#N/A</definedName>
+    <definedName name="Slicer_Region">#N/A</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
@@ -28,6 +31,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
       <x14:slicerCaches>
         <x14:slicerCache r:id="rId5"/>
+        <x14:slicerCache r:id="rId6"/>
+        <x14:slicerCache r:id="rId7"/>
+        <x14:slicerCache r:id="rId8"/>
       </x14:slicerCaches>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
@@ -44,7 +50,7 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="NlFk+p/PAWDUrEYESFxURzoSWKGV7010uFePnnXbbPA="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="NlFk+p/PAWDUrEYESFxURzoSWKGV7010uFePnnXbbPA="/>
     </ext>
   </extLst>
 </workbook>
@@ -73,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="124">
   <si>
     <t>Sale ID</t>
   </si>
@@ -429,37 +435,16 @@
     <t>Month</t>
   </si>
   <si>
-    <t>Jan</t>
-  </si>
-  <si>
     <t>Feb</t>
   </si>
   <si>
-    <t>Mar</t>
-  </si>
-  <si>
     <t>Apr</t>
   </si>
   <si>
-    <t>May</t>
-  </si>
-  <si>
     <t>Jun</t>
   </si>
   <si>
-    <t>Jul</t>
-  </si>
-  <si>
-    <t>Aug</t>
-  </si>
-  <si>
     <t>Sep</t>
-  </si>
-  <si>
-    <t>Oct</t>
-  </si>
-  <si>
-    <t>Nov</t>
   </si>
   <si>
     <t>Grand Total</t>
@@ -692,7 +677,1467 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="376">
+  <dxfs count="688">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <sz val="16"/>
+      </font>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
@@ -2515,8 +3960,242 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="12611100" y="373380"/>
-              <a:ext cx="1828800" cy="2466975"/>
+              <a:off x="11827528" y="372521"/>
+              <a:ext cx="1835347" cy="2481464"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>510540</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>510540</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>81915</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="3" name="Region">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72F9CACD-F9A6-7F9B-9C42-35BF8A08EAE0}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Region"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="13754315" y="380141"/>
+              <a:ext cx="1835239" cy="2481464"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>182880</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>426720</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>150495</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="4" name="Product Name">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E63E18B-4260-A3F3-D5C7-2031911F7C4B}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Product Name"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="11835148" y="2962570"/>
+              <a:ext cx="1835347" cy="2478995"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100"/>
+                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>510540</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>144780</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>510540</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>112395</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="5" name="Category">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B706E0E1-A769-25CA-267E-8217EC7AFD43}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="Category"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="13754315" y="2924470"/>
+              <a:ext cx="1835239" cy="2478995"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3115,7 +4794,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48B9EF5A-3213-4D38-979A-0805F2D584A7}" name="productcategory_sales" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="J3:K8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="J3:K5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0">
@@ -3147,7 +4826,21 @@
       </items>
     </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="11">
+        <item h="1" x="8"/>
+        <item h="1" x="0"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="2"/>
+        <item h="1" x="9"/>
+        <item h="1" x="5"/>
+        <item x="4"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
       <items count="5">
         <item x="1"/>
@@ -3163,18 +4856,9 @@
   <rowFields count="1">
     <field x="7"/>
   </rowFields>
-  <rowItems count="5">
+  <rowItems count="2">
     <i>
       <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -3187,22 +4871,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="351">
+    <format dxfId="663">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="352">
+    <format dxfId="664">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="353">
+    <format dxfId="665">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="354">
+    <format dxfId="666">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="355">
+    <format dxfId="667">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="356">
+    <format dxfId="668">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -3220,7 +4904,7 @@
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FC6400F2-21E4-469F-9AF0-F99BBDA61EFA}" name="productname_sales" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="G3:H14" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="G3:H5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0">
@@ -3254,56 +4938,37 @@
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
       <items count="11">
-        <item x="8"/>
-        <item x="0"/>
-        <item x="7"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="9"/>
-        <item x="5"/>
+        <item h="1" x="8"/>
+        <item h="1" x="0"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="2"/>
+        <item h="1" x="9"/>
+        <item h="1" x="5"/>
         <item x="4"/>
-        <item x="6"/>
-        <item x="1"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField dataField="1" compact="0" numFmtId="165" outline="0" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="6"/>
   </rowFields>
-  <rowItems count="11">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
+  <rowItems count="2">
     <i>
       <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
     </i>
     <i t="grand">
       <x/>
@@ -3316,22 +4981,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="357">
+    <format dxfId="669">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="358">
+    <format dxfId="670">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="359">
+    <format dxfId="671">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="360">
+    <format dxfId="672">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="361">
+    <format dxfId="673">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="362">
+    <format dxfId="674">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -3349,7 +5014,7 @@
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{71DD952B-FAC6-40F9-AA5F-00E82A8D09AD}" name="region_sales" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="D3:E9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="D3:E5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0">
@@ -3381,29 +5046,39 @@
       </items>
     </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="11">
+        <item h="1" x="8"/>
+        <item h="1" x="0"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="2"/>
+        <item h="1" x="9"/>
+        <item h="1" x="5"/>
+        <item x="4"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField dataField="1" compact="0" numFmtId="165" outline="0" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="4"/>
   </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
+  <rowItems count="2">
     <i>
       <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
     </i>
     <i t="grand">
       <x/>
@@ -3416,22 +5091,22 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="363">
+    <format dxfId="675">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="364">
+    <format dxfId="676">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="365">
+    <format dxfId="677">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="366">
+    <format dxfId="678">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0"/>
     </format>
-    <format dxfId="367">
+    <format dxfId="679">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="368">
+    <format dxfId="680">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -3449,7 +5124,7 @@
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{D9A74C0D-44F7-4925-B9F8-FF748A2C02BC}" name="month_sales" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="7" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="7" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="A3:B15" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
@@ -3470,49 +5145,59 @@
     </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="6">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="11">
+        <item h="1" x="8"/>
+        <item h="1" x="0"/>
+        <item h="1" x="7"/>
+        <item h="1" x="3"/>
+        <item h="1" x="2"/>
+        <item h="1" x="9"/>
+        <item h="1" x="5"/>
+        <item x="4"/>
+        <item h="1" x="6"/>
+        <item h="1" x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0">
+      <items count="5">
+        <item x="1"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField dataField="1" compact="0" numFmtId="165" outline="0" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="1"/>
   </rowFields>
-  <rowItems count="12">
-    <i>
-      <x/>
-    </i>
+  <rowItems count="5">
     <i>
       <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
     </i>
     <i>
       <x v="3"/>
     </i>
     <i>
-      <x v="4"/>
-    </i>
-    <i>
       <x v="5"/>
     </i>
     <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
       <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x v="10"/>
     </i>
     <i t="grand">
       <x/>
@@ -3525,29 +5210,29 @@
     <dataField name="Total Sale" fld="9" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
   <formats count="7">
-    <format dxfId="375">
+    <format dxfId="687">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="374">
+    <format dxfId="686">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="373">
+    <format dxfId="685">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="372">
+    <format dxfId="684">
       <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="371">
+    <format dxfId="683">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="1" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="370">
+    <format dxfId="682">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="369">
+    <format dxfId="681">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -3574,17 +5259,87 @@
   <data>
     <tabular pivotCacheId="1167224161">
       <items count="11">
-        <i x="0" s="1"/>
         <i x="1" s="1"/>
-        <i x="2" s="1"/>
         <i x="3" s="1"/>
+        <i x="5" s="1"/>
+        <i x="8" s="1"/>
+        <i x="0" s="1" nd="1"/>
+        <i x="2" s="1" nd="1"/>
+        <i x="4" s="1" nd="1"/>
+        <i x="6" s="1" nd="1"/>
+        <i x="7" s="1" nd="1"/>
+        <i x="9" s="1" nd="1"/>
+        <i x="10" s="1" nd="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache2.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Region" xr10:uid="{8196A1D7-AABC-4F4C-955B-D3EB0E4CFE36}" sourceName="Region">
+  <pivotTables>
+    <pivotTable tabId="4" name="region_sales"/>
+    <pivotTable tabId="4" name="month_sales"/>
+    <pivotTable tabId="4" name="productcategory_sales"/>
+    <pivotTable tabId="4" name="productname_sales"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1167224161">
+      <items count="5">
         <i x="4" s="1"/>
-        <i x="5" s="1"/>
-        <i x="6" s="1"/>
-        <i x="7" s="1"/>
-        <i x="8" s="1"/>
-        <i x="9" s="1"/>
-        <i x="10" s="1"/>
+        <i x="1" s="1" nd="1"/>
+        <i x="0" s="1" nd="1"/>
+        <i x="3" s="1" nd="1"/>
+        <i x="2" s="1" nd="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache3.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Product_Name" xr10:uid="{D90D85BC-9D3B-434A-9341-ADCF5A381D75}" sourceName="Product Name">
+  <pivotTables>
+    <pivotTable tabId="4" name="productname_sales"/>
+    <pivotTable tabId="4" name="month_sales"/>
+    <pivotTable tabId="4" name="productcategory_sales"/>
+    <pivotTable tabId="4" name="region_sales"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1167224161">
+      <items count="10">
+        <i x="8"/>
+        <i x="0"/>
+        <i x="7"/>
+        <i x="3"/>
+        <i x="2"/>
+        <i x="9"/>
+        <i x="5"/>
+        <i x="4" s="1"/>
+        <i x="6"/>
+        <i x="1"/>
+      </items>
+    </tabular>
+  </data>
+</slicerCacheDefinition>
+</file>
+
+<file path=xl/slicerCaches/slicerCache4.xml><?xml version="1.0" encoding="utf-8"?>
+<slicerCacheDefinition xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10" name="Slicer_Category" xr10:uid="{6E1D617A-7BB5-4333-9A19-298613B7F331}" sourceName="Category">
+  <pivotTables>
+    <pivotTable tabId="4" name="productname_sales"/>
+    <pivotTable tabId="4" name="month_sales"/>
+    <pivotTable tabId="4" name="productcategory_sales"/>
+    <pivotTable tabId="4" name="region_sales"/>
+  </pivotTables>
+  <data>
+    <tabular pivotCacheId="1167224161">
+      <items count="4">
+        <i x="1" s="1"/>
+        <i x="0" s="1" nd="1"/>
+        <i x="2" s="1" nd="1"/>
+        <i x="3" s="1" nd="1"/>
       </items>
     </tabular>
   </data>
@@ -3594,6 +5349,9 @@
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
   <slicer name="Month" xr10:uid="{8F227F2F-9E99-497F-B577-006C74605616}" cache="Slicer_Month" caption="Month" rowHeight="234950"/>
+  <slicer name="Region" xr10:uid="{017C1462-0B3D-447B-8DB5-D271F4DF779F}" cache="Slicer_Region" caption="Region" rowHeight="234950"/>
+  <slicer name="Product Name" xr10:uid="{7CCC28DC-0441-46BA-9DDC-D3904E810648}" cache="Slicer_Product_Name" caption="Product Name" rowHeight="234950"/>
+  <slicer name="Category" xr10:uid="{2F44CD1F-B498-4A4B-9353-9DE6282BCC6A}" cache="Slicer_Category" caption="Category" rowHeight="234950"/>
 </slicers>
 </file>
 
@@ -3798,15 +5556,15 @@
   <dimension ref="A3:K19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.21875" customWidth="1"/>
-    <col min="10" max="10" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3815,25 +5573,25 @@
         <v>117</v>
       </c>
       <c r="B3" s="22" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="D3" s="21" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="22" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="G3" s="21" t="s">
         <v>5</v>
       </c>
       <c r="H3" s="22" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="J3" s="21" t="s">
         <v>6</v>
       </c>
       <c r="K3" s="22" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="21" x14ac:dyDescent="0.4">
@@ -3841,25 +5599,25 @@
         <v>118</v>
       </c>
       <c r="B4" s="23">
-        <v>359800</v>
+        <v>28000</v>
       </c>
       <c r="D4" s="22" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="E4" s="23">
-        <v>184500</v>
+        <v>143500</v>
       </c>
       <c r="G4" s="22" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="H4" s="23">
-        <v>138600</v>
+        <v>143500</v>
       </c>
       <c r="J4" s="22" t="s">
         <v>20</v>
       </c>
       <c r="K4" s="23">
-        <v>208400</v>
+        <v>143500</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="21" x14ac:dyDescent="0.4">
@@ -3867,25 +5625,25 @@
         <v>119</v>
       </c>
       <c r="B5" s="23">
-        <v>326000</v>
+        <v>24500</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>12</v>
+        <v>122</v>
       </c>
       <c r="E5" s="23">
-        <v>4061000</v>
+        <v>143500</v>
       </c>
       <c r="G5" s="22" t="s">
-        <v>13</v>
+        <v>122</v>
       </c>
       <c r="H5" s="23">
-        <v>3025000</v>
+        <v>143500</v>
       </c>
       <c r="J5" s="22" t="s">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="K5" s="23">
-        <v>3621500</v>
+        <v>143500</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="21" x14ac:dyDescent="0.4">
@@ -3893,25 +5651,7 @@
         <v>120</v>
       </c>
       <c r="B6" s="23">
-        <v>925200</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" s="23">
-        <v>282100</v>
-      </c>
-      <c r="G6" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="23">
-        <v>448000</v>
-      </c>
-      <c r="J6" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="K6" s="23">
-        <v>1609600</v>
+        <v>52500</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="21" x14ac:dyDescent="0.4">
@@ -3919,25 +5659,7 @@
         <v>121</v>
       </c>
       <c r="B7" s="23">
-        <v>102350</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="23">
-        <v>452950</v>
-      </c>
-      <c r="G7" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="23">
-        <v>4950</v>
-      </c>
-      <c r="J7" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="K7" s="23">
-        <v>4950</v>
+        <v>38500</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="21" x14ac:dyDescent="0.4">
@@ -3945,125 +5667,16 @@
         <v>122</v>
       </c>
       <c r="B8" s="23">
-        <v>858600</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="23">
-        <v>463900</v>
-      </c>
-      <c r="G8" s="22" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" s="23">
-        <v>435000</v>
-      </c>
-      <c r="J8" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="K8" s="23">
-        <v>5444450</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="21" x14ac:dyDescent="0.4">
-      <c r="A9" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="B9" s="23">
-        <v>284100</v>
-      </c>
-      <c r="D9" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="E9" s="23">
-        <v>5444450</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="H9" s="23">
-        <v>28900</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="21" x14ac:dyDescent="0.4">
-      <c r="A10" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="B10" s="23">
-        <v>765350</v>
-      </c>
-      <c r="G10" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="H10" s="23">
-        <v>1036000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="21" x14ac:dyDescent="0.4">
-      <c r="A11" s="22" t="s">
-        <v>125</v>
-      </c>
-      <c r="B11" s="23">
-        <v>721600</v>
-      </c>
-      <c r="G11" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="H11" s="23">
         <v>143500</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="21" x14ac:dyDescent="0.4">
-      <c r="A12" s="22" t="s">
-        <v>126</v>
-      </c>
-      <c r="B12" s="23">
-        <v>276000</v>
-      </c>
-      <c r="G12" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="H12" s="23">
-        <v>148500</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="21" x14ac:dyDescent="0.4">
-      <c r="A13" s="22" t="s">
-        <v>127</v>
-      </c>
-      <c r="B13" s="23">
-        <v>165450</v>
-      </c>
-      <c r="G13" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="H13" s="23">
-        <v>36000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="21" x14ac:dyDescent="0.4">
-      <c r="A14" s="22" t="s">
-        <v>128</v>
-      </c>
-      <c r="B14" s="23">
-        <v>660000</v>
-      </c>
-      <c r="G14" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="H14" s="23">
-        <v>5444450</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="21" x14ac:dyDescent="0.4">
-      <c r="A15" s="22" t="s">
-        <v>129</v>
-      </c>
-      <c r="B15" s="23">
-        <v>5444450</v>
-      </c>
-    </row>
+    <row r="9" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="10" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="11" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="12" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="13" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="14" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
+    <row r="15" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
     <row r="16" spans="1:11" ht="21" x14ac:dyDescent="0.4"/>
     <row r="17" ht="21" x14ac:dyDescent="0.4"/>
     <row r="18" ht="21" x14ac:dyDescent="0.4"/>

</xml_diff>